<commit_message>
feat: rename glaze "Men lam thường" to "Men lam"
Customers misread "thường" on quotes. The server renames the old glaze
in stored data at startup (after a snapshot) and on every write, so old
backups and browser data cannot bring it back.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Bang_gia_mau_Gom_Vu_Gia.xlsx
+++ b/data/Bang_gia_mau_Gom_Vu_Gia.xlsx
@@ -521,7 +521,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Sheet “Bảng giá 2 cột giá”: giống bố cục PDF, giá Men lam thường và Men lam vẽ vàng nằm ở 2 cột. Khi nhập, chọn cả 2 cột giá để ứng dụng tách thành biến thể.</t>
+          <t>Sheet “Bảng giá 2 cột giá”: giống bố cục PDF, giá Men lam và Men lam vẽ vàng nằm ở 2 cột. Khi nhập, chọn cả 2 cột giá để ứng dụng tách thành biến thể.</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -802,7 +802,7 @@
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -886,7 +886,7 @@
       <c r="E9" s="8" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -1062,7 +1062,7 @@
       <c r="E13" s="8" t="inlineStr"/>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -1146,7 +1146,7 @@
       <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -1226,7 +1226,7 @@
       <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -2802,7 +2802,7 @@
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G49" s="8" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G55" s="8" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr">
@@ -3502,7 +3502,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G65" s="8" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G67" s="8" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G71" s="8" t="inlineStr">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G73" s="8" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G75" s="8" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G77" s="8" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="F79" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G79" s="8" t="inlineStr">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G81" s="8" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G83" s="8" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G85" s="8" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="F87" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G87" s="8" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G89" s="8" t="inlineStr">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G91" s="8" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="F93" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G93" s="8" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G95" s="8" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="F105" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G105" s="8" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G107" s="8" t="inlineStr">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="F109" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G109" s="8" t="inlineStr">
@@ -5854,7 +5854,7 @@
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G111" s="8" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G113" s="8" t="inlineStr">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G115" s="8" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G117" s="8" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G119" s="8" t="inlineStr">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G121" s="8" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="F123" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G123" s="8" t="inlineStr">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="F125" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G125" s="8" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="F127" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G127" s="8" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="F129" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G129" s="8" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="F131" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G131" s="8" t="inlineStr">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="F133" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G133" s="8" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="F135" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G135" s="8" t="inlineStr">
@@ -7154,7 +7154,7 @@
       </c>
       <c r="F137" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G137" s="8" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="F139" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G139" s="8" t="inlineStr">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="F141" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G141" s="8" t="inlineStr">
@@ -7454,7 +7454,7 @@
       </c>
       <c r="F143" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G143" s="8" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="F145" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G145" s="8" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="F147" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G147" s="8" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="F149" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G149" s="8" t="inlineStr">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="F151" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G151" s="8" t="inlineStr">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="F153" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G153" s="8" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="F155" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G155" s="8" t="inlineStr">
@@ -8150,7 +8150,7 @@
       <c r="E157" s="8" t="inlineStr"/>
       <c r="F157" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G157" s="8" t="inlineStr">
@@ -8242,7 +8242,7 @@
       <c r="E159" s="8" t="inlineStr"/>
       <c r="F159" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G159" s="8" t="inlineStr">
@@ -8334,7 +8334,7 @@
       <c r="E161" s="8" t="inlineStr"/>
       <c r="F161" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G161" s="8" t="inlineStr">
@@ -8426,7 +8426,7 @@
       <c r="E163" s="8" t="inlineStr"/>
       <c r="F163" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G163" s="8" t="inlineStr">
@@ -8518,7 +8518,7 @@
       <c r="E165" s="8" t="inlineStr"/>
       <c r="F165" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G165" s="8" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="F167" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G167" s="8" t="inlineStr">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="F169" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G169" s="8" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="F171" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G171" s="8" t="inlineStr">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="F173" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G173" s="8" t="inlineStr">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="F175" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G175" s="8" t="inlineStr">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="F177" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G177" s="8" t="inlineStr">
@@ -9214,7 +9214,7 @@
       </c>
       <c r="F179" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G179" s="8" t="inlineStr">
@@ -9314,7 +9314,7 @@
       </c>
       <c r="F181" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G181" s="8" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="F183" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G183" s="8" t="inlineStr">
@@ -9514,7 +9514,7 @@
       </c>
       <c r="F185" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G185" s="8" t="inlineStr">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="F187" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G187" s="8" t="inlineStr">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="F189" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G189" s="8" t="inlineStr">
@@ -9810,7 +9810,7 @@
       <c r="E191" s="8" t="inlineStr"/>
       <c r="F191" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G191" s="8" t="inlineStr">
@@ -9898,7 +9898,7 @@
       <c r="E193" s="8" t="inlineStr"/>
       <c r="F193" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G193" s="8" t="inlineStr">
@@ -9984,7 +9984,7 @@
       <c r="E195" s="8" t="inlineStr"/>
       <c r="F195" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G195" s="8" t="inlineStr">
@@ -10068,7 +10068,7 @@
       <c r="E197" s="8" t="inlineStr"/>
       <c r="F197" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G197" s="8" t="inlineStr">
@@ -10148,7 +10148,7 @@
       <c r="E199" s="8" t="inlineStr"/>
       <c r="F199" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G199" s="8" t="inlineStr">
@@ -10236,7 +10236,7 @@
       <c r="E201" s="8" t="inlineStr"/>
       <c r="F201" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G201" s="8" t="inlineStr">
@@ -10332,7 +10332,7 @@
       </c>
       <c r="F203" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G203" s="8" t="inlineStr">
@@ -10432,7 +10432,7 @@
       </c>
       <c r="F205" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G205" s="8" t="inlineStr">
@@ -10528,7 +10528,7 @@
       <c r="E207" s="8" t="inlineStr"/>
       <c r="F207" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G207" s="8" t="inlineStr">
@@ -10620,7 +10620,7 @@
       <c r="E209" s="8" t="inlineStr"/>
       <c r="F209" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G209" s="8" t="inlineStr">
@@ -10704,7 +10704,7 @@
       <c r="E211" s="8" t="inlineStr"/>
       <c r="F211" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G211" s="8" t="inlineStr">
@@ -10784,7 +10784,7 @@
       <c r="E213" s="8" t="inlineStr"/>
       <c r="F213" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G213" s="8" t="inlineStr">
@@ -10876,7 +10876,7 @@
       </c>
       <c r="F215" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G215" s="8" t="inlineStr">
@@ -10976,7 +10976,7 @@
       </c>
       <c r="F217" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G217" s="8" t="inlineStr">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G219" s="8" t="inlineStr">
@@ -11172,7 +11172,7 @@
       <c r="E221" s="8" t="inlineStr"/>
       <c r="F221" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G221" s="8" t="inlineStr">
@@ -11268,7 +11268,7 @@
       </c>
       <c r="F223" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G223" s="8" t="inlineStr">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="F225" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G225" s="8" t="inlineStr">
@@ -11464,7 +11464,7 @@
       <c r="E227" s="8" t="inlineStr"/>
       <c r="F227" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G227" s="8" t="inlineStr">
@@ -11552,7 +11552,7 @@
       <c r="E229" s="8" t="inlineStr"/>
       <c r="F229" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G229" s="8" t="inlineStr">
@@ -11628,7 +11628,7 @@
       <c r="E231" s="8" t="inlineStr"/>
       <c r="F231" s="7" t="inlineStr">
         <is>
-          <t>Men lam thường</t>
+          <t>Men lam</t>
         </is>
       </c>
       <c r="G231" s="8" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="G1" s="6" t="inlineStr">
         <is>
-          <t>Giá Men lam thường</t>
+          <t>Giá Men lam</t>
         </is>
       </c>
       <c r="H1" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat: update price list and sync prices on deploy
Apply the new men lam price sheet (all men lam prices, two vàng kim
prices) and add four loose HMT set items. On startup the server applies
data/pdf_data.json by product code once per file version, after taking a
snapshot; it never deletes products or touches saved templates/quotes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Bang_gia_mau_Gom_Vu_Gia.xlsx
+++ b/data/Bang_gia_mau_Gom_Vu_Gia.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng giá 2 cột giá" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bảng giá theo biến thể'!$A$4:$J$232</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bảng giá theo biến thể'!$A$4:$J$240</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J232"/>
+  <dimension ref="A1:J240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="H5" s="9" t="n">
-        <v>19000000</v>
+        <v>23000000</v>
       </c>
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="8" t="inlineStr">
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="H6" s="9" t="n">
-        <v>38800000</v>
+        <v>38600000</v>
       </c>
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="8" t="inlineStr">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="H7" s="9" t="n">
-        <v>17500000</v>
+        <v>21500000</v>
       </c>
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="8" t="inlineStr">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="H9" s="9" t="n">
-        <v>11000000</v>
+        <v>13500000</v>
       </c>
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="8" t="inlineStr">
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="H11" s="9" t="n">
-        <v>16500000</v>
+        <v>20500000</v>
       </c>
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="8" t="inlineStr">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="H12" s="9" t="n">
-        <v>37500000</v>
+        <v>37600000</v>
       </c>
       <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="8" t="inlineStr">
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="H13" s="9" t="n">
-        <v>15500000</v>
+        <v>19000000</v>
       </c>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="H15" s="9" t="n">
-        <v>8800000</v>
+        <v>11000000</v>
       </c>
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="8" t="inlineStr">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="H17" s="9" t="n">
-        <v>1100000</v>
+        <v>1500000</v>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="H19" s="9" t="n">
-        <v>6600000</v>
+        <v>8000000</v>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="H21" s="9" t="n">
-        <v>2640000</v>
+        <v>3000000</v>
       </c>
       <c r="I21" s="7" t="inlineStr"/>
       <c r="J21" s="8" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="H23" s="9" t="n">
-        <v>2200000</v>
+        <v>2650000</v>
       </c>
       <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="8" t="inlineStr">
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="H25" s="9" t="n">
-        <v>1200000</v>
+        <v>1450000</v>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="H27" s="9" t="n">
-        <v>700000</v>
+        <v>850000</v>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="H29" s="9" t="n">
-        <v>550000</v>
+        <v>660000</v>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="H31" s="9" t="n">
-        <v>440000</v>
+        <v>530000</v>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="H33" s="9" t="n">
-        <v>400000</v>
+        <v>480000</v>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="H35" s="9" t="n">
-        <v>265000</v>
+        <v>320000</v>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="H37" s="9" t="n">
-        <v>210000</v>
+        <v>250000</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
@@ -2311,7 +2311,7 @@
         </is>
       </c>
       <c r="H39" s="9" t="n">
-        <v>2200000</v>
+        <v>2650000</v>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
@@ -2411,7 +2411,7 @@
         </is>
       </c>
       <c r="H41" s="9" t="n">
-        <v>1000000</v>
+        <v>1200000</v>
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
@@ -2511,7 +2511,7 @@
         </is>
       </c>
       <c r="H43" s="9" t="n">
-        <v>800000</v>
+        <v>960000</v>
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="H45" s="9" t="n">
-        <v>550000</v>
+        <v>660000</v>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="H47" s="9" t="n">
-        <v>450000</v>
+        <v>550000</v>
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
@@ -2811,7 +2811,7 @@
         </is>
       </c>
       <c r="H49" s="9" t="n">
-        <v>350000</v>
+        <v>420000</v>
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="H51" s="9" t="n">
-        <v>1100000</v>
+        <v>1320000</v>
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
@@ -3011,7 +3011,7 @@
         </is>
       </c>
       <c r="H53" s="9" t="n">
-        <v>650000</v>
+        <v>780000</v>
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
         </is>
       </c>
       <c r="H55" s="9" t="n">
-        <v>510000</v>
+        <v>620000</v>
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="H57" s="9" t="n">
-        <v>400000</v>
+        <v>480000</v>
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="H59" s="9" t="n">
-        <v>310000</v>
+        <v>380000</v>
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="H61" s="9" t="n">
-        <v>230000</v>
+        <v>280000</v>
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="H63" s="9" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="H65" s="9" t="n">
-        <v>2100000</v>
+        <v>2500000</v>
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
@@ -3711,7 +3711,7 @@
         </is>
       </c>
       <c r="H67" s="9" t="n">
-        <v>880000</v>
+        <v>1100000</v>
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
@@ -3811,7 +3811,7 @@
         </is>
       </c>
       <c r="H69" s="9" t="n">
-        <v>770000</v>
+        <v>930000</v>
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
@@ -3911,7 +3911,7 @@
         </is>
       </c>
       <c r="H71" s="9" t="n">
-        <v>660000</v>
+        <v>800000</v>
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="H73" s="9" t="n">
-        <v>550000</v>
+        <v>660000</v>
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
@@ -4111,7 +4111,7 @@
         </is>
       </c>
       <c r="H75" s="9" t="n">
-        <v>270000</v>
+        <v>325000</v>
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="H77" s="9" t="n">
-        <v>230000</v>
+        <v>280000</v>
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
@@ -4299,7 +4299,7 @@
         </is>
       </c>
       <c r="H79" s="9" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
@@ -4391,7 +4391,7 @@
         </is>
       </c>
       <c r="H81" s="9" t="n">
-        <v>290000</v>
+        <v>350000</v>
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
         </is>
       </c>
       <c r="H83" s="9" t="n">
-        <v>320000</v>
+        <v>380000</v>
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
@@ -4575,7 +4575,7 @@
         </is>
       </c>
       <c r="H85" s="9" t="n">
-        <v>450000</v>
+        <v>540000</v>
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
@@ -4667,7 +4667,7 @@
         </is>
       </c>
       <c r="H87" s="9" t="n">
-        <v>480000</v>
+        <v>580000</v>
       </c>
       <c r="I87" s="7" t="inlineStr">
         <is>
@@ -4763,7 +4763,7 @@
         </is>
       </c>
       <c r="H89" s="9" t="n">
-        <v>750000</v>
+        <v>900000</v>
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
@@ -4863,7 +4863,7 @@
         </is>
       </c>
       <c r="H91" s="9" t="n">
-        <v>1050000</v>
+        <v>1250000</v>
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
@@ -4963,7 +4963,7 @@
         </is>
       </c>
       <c r="H93" s="9" t="n">
-        <v>980000</v>
+        <v>1200000</v>
       </c>
       <c r="I93" s="7" t="inlineStr">
         <is>
@@ -5063,7 +5063,7 @@
         </is>
       </c>
       <c r="H95" s="9" t="n">
-        <v>2200000</v>
+        <v>2650000</v>
       </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
@@ -5163,7 +5163,7 @@
         </is>
       </c>
       <c r="H97" s="9" t="n">
-        <v>3300000</v>
+        <v>4000000</v>
       </c>
       <c r="I97" s="7" t="inlineStr">
         <is>
@@ -5263,7 +5263,7 @@
         </is>
       </c>
       <c r="H99" s="9" t="n">
-        <v>350000</v>
+        <v>420000</v>
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
@@ -5363,7 +5363,7 @@
         </is>
       </c>
       <c r="H101" s="9" t="n">
-        <v>280000</v>
+        <v>340000</v>
       </c>
       <c r="I101" s="7" t="inlineStr">
         <is>
@@ -5463,7 +5463,7 @@
         </is>
       </c>
       <c r="H103" s="9" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="I103" s="7" t="inlineStr">
         <is>
@@ -5563,7 +5563,7 @@
         </is>
       </c>
       <c r="H105" s="9" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="I105" s="7" t="inlineStr">
         <is>
@@ -5663,7 +5663,7 @@
         </is>
       </c>
       <c r="H107" s="9" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="I107" s="7" t="inlineStr">
         <is>
@@ -5763,7 +5763,7 @@
         </is>
       </c>
       <c r="H109" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I109" s="7" t="inlineStr">
         <is>
@@ -5863,7 +5863,7 @@
         </is>
       </c>
       <c r="H111" s="9" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="I111" s="7" t="inlineStr">
         <is>
@@ -5963,7 +5963,7 @@
         </is>
       </c>
       <c r="H113" s="9" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="I113" s="7" t="inlineStr">
         <is>
@@ -6063,7 +6063,7 @@
         </is>
       </c>
       <c r="H115" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I115" s="7" t="inlineStr">
         <is>
@@ -6163,7 +6163,7 @@
         </is>
       </c>
       <c r="H117" s="9" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="I117" s="7" t="inlineStr">
         <is>
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="H119" s="9" t="n">
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="I119" s="7" t="inlineStr">
         <is>
@@ -6363,7 +6363,7 @@
         </is>
       </c>
       <c r="H121" s="9" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="I121" s="7" t="inlineStr">
         <is>
@@ -6463,7 +6463,7 @@
         </is>
       </c>
       <c r="H123" s="9" t="n">
-        <v>910000</v>
+        <v>1100000</v>
       </c>
       <c r="I123" s="7" t="inlineStr">
         <is>
@@ -6563,7 +6563,7 @@
         </is>
       </c>
       <c r="H125" s="9" t="n">
-        <v>785000</v>
+        <v>950000</v>
       </c>
       <c r="I125" s="7" t="inlineStr">
         <is>
@@ -6663,7 +6663,7 @@
         </is>
       </c>
       <c r="H127" s="9" t="n">
-        <v>660000</v>
+        <v>800000</v>
       </c>
       <c r="I127" s="7" t="inlineStr">
         <is>
@@ -6763,7 +6763,7 @@
         </is>
       </c>
       <c r="H129" s="9" t="n">
-        <v>575000</v>
+        <v>700000</v>
       </c>
       <c r="I129" s="7" t="inlineStr">
         <is>
@@ -6863,7 +6863,7 @@
         </is>
       </c>
       <c r="H131" s="9" t="n">
-        <v>450000</v>
+        <v>550000</v>
       </c>
       <c r="I131" s="7" t="inlineStr">
         <is>
@@ -6963,7 +6963,7 @@
         </is>
       </c>
       <c r="H133" s="9" t="n">
-        <v>330000</v>
+        <v>400000</v>
       </c>
       <c r="I133" s="7" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="H135" s="9" t="n">
-        <v>280000</v>
+        <v>350000</v>
       </c>
       <c r="I135" s="7" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         </is>
       </c>
       <c r="H137" s="9" t="n">
-        <v>240000</v>
+        <v>300000</v>
       </c>
       <c r="I137" s="7" t="inlineStr">
         <is>
@@ -7263,7 +7263,7 @@
         </is>
       </c>
       <c r="H139" s="9" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="I139" s="7" t="inlineStr">
         <is>
@@ -7363,7 +7363,7 @@
         </is>
       </c>
       <c r="H141" s="9" t="n">
-        <v>1050000</v>
+        <v>1260000</v>
       </c>
       <c r="I141" s="7" t="inlineStr">
         <is>
@@ -7463,7 +7463,7 @@
         </is>
       </c>
       <c r="H143" s="9" t="n">
-        <v>890000</v>
+        <v>1100000</v>
       </c>
       <c r="I143" s="7" t="inlineStr">
         <is>
@@ -7563,7 +7563,7 @@
         </is>
       </c>
       <c r="H145" s="9" t="n">
-        <v>750000</v>
+        <v>900000</v>
       </c>
       <c r="I145" s="7" t="inlineStr">
         <is>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="H147" s="9" t="n">
-        <v>620000</v>
+        <v>750000</v>
       </c>
       <c r="I147" s="7" t="inlineStr">
         <is>
@@ -7763,7 +7763,7 @@
         </is>
       </c>
       <c r="H149" s="9" t="n">
-        <v>490000</v>
+        <v>600000</v>
       </c>
       <c r="I149" s="7" t="inlineStr">
         <is>
@@ -7863,7 +7863,7 @@
         </is>
       </c>
       <c r="H151" s="9" t="n">
-        <v>390000</v>
+        <v>480000</v>
       </c>
       <c r="I151" s="7" t="inlineStr">
         <is>
@@ -7963,7 +7963,7 @@
         </is>
       </c>
       <c r="H153" s="9" t="n">
-        <v>330000</v>
+        <v>400000</v>
       </c>
       <c r="I153" s="7" t="inlineStr">
         <is>
@@ -8063,7 +8063,7 @@
         </is>
       </c>
       <c r="H155" s="9" t="n">
-        <v>260000</v>
+        <v>320000</v>
       </c>
       <c r="I155" s="7" t="inlineStr">
         <is>
@@ -8159,7 +8159,7 @@
         </is>
       </c>
       <c r="H157" s="9" t="n">
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="I157" s="7" t="inlineStr">
         <is>
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="H159" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I159" s="7" t="inlineStr">
         <is>
@@ -8343,7 +8343,7 @@
         </is>
       </c>
       <c r="H161" s="9" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="I161" s="7" t="inlineStr">
         <is>
@@ -8435,7 +8435,7 @@
         </is>
       </c>
       <c r="H163" s="9" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="I163" s="7" t="inlineStr">
         <is>
@@ -8527,7 +8527,7 @@
         </is>
       </c>
       <c r="H165" s="9" t="n">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="I165" s="7" t="inlineStr">
         <is>
@@ -8623,7 +8623,7 @@
         </is>
       </c>
       <c r="H167" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I167" s="7" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
         </is>
       </c>
       <c r="H169" s="9" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="I169" s="7" t="inlineStr">
         <is>
@@ -8823,7 +8823,7 @@
         </is>
       </c>
       <c r="H171" s="9" t="n">
-        <v>200000</v>
+        <v>240000</v>
       </c>
       <c r="I171" s="7" t="inlineStr">
         <is>
@@ -8923,7 +8923,7 @@
         </is>
       </c>
       <c r="H173" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I173" s="7" t="inlineStr">
         <is>
@@ -9023,7 +9023,7 @@
         </is>
       </c>
       <c r="H175" s="9" t="n">
-        <v>165000</v>
+        <v>200000</v>
       </c>
       <c r="I175" s="7" t="inlineStr">
         <is>
@@ -9123,7 +9123,7 @@
         </is>
       </c>
       <c r="H177" s="9" t="n">
-        <v>135000</v>
+        <v>165000</v>
       </c>
       <c r="I177" s="7" t="inlineStr">
         <is>
@@ -9223,7 +9223,7 @@
         </is>
       </c>
       <c r="H179" s="9" t="n">
-        <v>165000</v>
+        <v>200000</v>
       </c>
       <c r="I179" s="7" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
         </is>
       </c>
       <c r="H181" s="9" t="n">
-        <v>135000</v>
+        <v>160000</v>
       </c>
       <c r="I181" s="7" t="inlineStr">
         <is>
@@ -9423,7 +9423,7 @@
         </is>
       </c>
       <c r="H183" s="9" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="I183" s="7" t="inlineStr">
         <is>
@@ -9523,7 +9523,7 @@
         </is>
       </c>
       <c r="H185" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I185" s="7" t="inlineStr">
         <is>
@@ -9623,7 +9623,7 @@
         </is>
       </c>
       <c r="H187" s="9" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="I187" s="7" t="inlineStr">
         <is>
@@ -9723,7 +9723,7 @@
         </is>
       </c>
       <c r="H189" s="9" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="I189" s="7" t="inlineStr">
         <is>
@@ -9819,7 +9819,7 @@
         </is>
       </c>
       <c r="H191" s="9" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="I191" s="7" t="inlineStr">
         <is>
@@ -9907,7 +9907,7 @@
         </is>
       </c>
       <c r="H193" s="9" t="n">
-        <v>22000</v>
+        <v>28000</v>
       </c>
       <c r="I193" s="7" t="inlineStr">
         <is>
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="H195" s="9" t="n">
-        <v>200000</v>
+        <v>270000</v>
       </c>
       <c r="I195" s="7" t="inlineStr"/>
       <c r="J195" s="8" t="inlineStr">
@@ -10077,7 +10077,7 @@
         </is>
       </c>
       <c r="H197" s="9" t="n">
-        <v>165000</v>
+        <v>200000</v>
       </c>
       <c r="I197" s="7" t="inlineStr"/>
       <c r="J197" s="8" t="inlineStr">
@@ -10157,7 +10157,7 @@
         </is>
       </c>
       <c r="H199" s="9" t="n">
-        <v>22000</v>
+        <v>28000</v>
       </c>
       <c r="I199" s="7" t="inlineStr">
         <is>
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="H201" s="9" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="I201" s="7" t="inlineStr">
         <is>
@@ -10341,7 +10341,7 @@
         </is>
       </c>
       <c r="H203" s="9" t="n">
-        <v>88000</v>
+        <v>110000</v>
       </c>
       <c r="I203" s="7" t="inlineStr">
         <is>
@@ -10441,7 +10441,7 @@
         </is>
       </c>
       <c r="H205" s="9" t="n">
-        <v>66000</v>
+        <v>80000</v>
       </c>
       <c r="I205" s="7" t="inlineStr">
         <is>
@@ -10537,7 +10537,7 @@
         </is>
       </c>
       <c r="H207" s="9" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="I207" s="7" t="inlineStr">
         <is>
@@ -10629,7 +10629,7 @@
         </is>
       </c>
       <c r="H209" s="9" t="n">
-        <v>265000</v>
+        <v>320000</v>
       </c>
       <c r="I209" s="7" t="inlineStr"/>
       <c r="J209" s="8" t="inlineStr">
@@ -10713,7 +10713,7 @@
         </is>
       </c>
       <c r="H211" s="9" t="n">
-        <v>400000</v>
+        <v>480000</v>
       </c>
       <c r="I211" s="7" t="inlineStr"/>
       <c r="J211" s="8" t="inlineStr">
@@ -10793,7 +10793,7 @@
         </is>
       </c>
       <c r="H213" s="9" t="n">
-        <v>22000</v>
+        <v>26000</v>
       </c>
       <c r="I213" s="7" t="inlineStr">
         <is>
@@ -10885,7 +10885,7 @@
         </is>
       </c>
       <c r="H215" s="9" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="I215" s="7" t="inlineStr">
         <is>
@@ -10985,7 +10985,7 @@
         </is>
       </c>
       <c r="H217" s="9" t="n">
-        <v>88000</v>
+        <v>105000</v>
       </c>
       <c r="I217" s="7" t="inlineStr">
         <is>
@@ -11085,7 +11085,7 @@
         </is>
       </c>
       <c r="H219" s="9" t="n">
-        <v>66000</v>
+        <v>80000</v>
       </c>
       <c r="I219" s="7" t="inlineStr">
         <is>
@@ -11181,7 +11181,7 @@
         </is>
       </c>
       <c r="H221" s="9" t="n">
-        <v>45000</v>
+        <v>55000</v>
       </c>
       <c r="I221" s="7" t="inlineStr">
         <is>
@@ -11277,7 +11277,7 @@
         </is>
       </c>
       <c r="H223" s="9" t="n">
-        <v>1650000</v>
+        <v>2000000</v>
       </c>
       <c r="I223" s="7" t="inlineStr">
         <is>
@@ -11377,7 +11377,7 @@
         </is>
       </c>
       <c r="H225" s="9" t="n">
-        <v>1320000</v>
+        <v>1600000</v>
       </c>
       <c r="I225" s="7" t="inlineStr">
         <is>
@@ -11473,7 +11473,7 @@
         </is>
       </c>
       <c r="H227" s="9" t="n">
-        <v>660000</v>
+        <v>800000</v>
       </c>
       <c r="I227" s="7" t="inlineStr">
         <is>
@@ -11561,7 +11561,7 @@
         </is>
       </c>
       <c r="H229" s="9" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="I229" s="7" t="inlineStr"/>
       <c r="J229" s="8" t="inlineStr">
@@ -11637,7 +11637,7 @@
         </is>
       </c>
       <c r="H231" s="9" t="n">
-        <v>135000</v>
+        <v>160000</v>
       </c>
       <c r="I231" s="7" t="inlineStr"/>
       <c r="J231" s="8" t="inlineStr">
@@ -11686,8 +11686,368 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" s="7" t="inlineStr">
+        <is>
+          <t>DA07-ML</t>
+        </is>
+      </c>
+      <c r="B233" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C233" s="7" t="inlineStr">
+        <is>
+          <t>Bát tô canh vẽ tay</t>
+        </is>
+      </c>
+      <c r="D233" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E233" s="8" t="inlineStr"/>
+      <c r="F233" s="7" t="inlineStr">
+        <is>
+          <t>Men lam</t>
+        </is>
+      </c>
+      <c r="G233" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H233" s="9" t="n">
+        <v>686400</v>
+      </c>
+      <c r="I233" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+      <c r="J233" s="8" t="inlineStr">
+        <is>
+          <t>Đang dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="7" t="inlineStr">
+        <is>
+          <t>DA07-VV</t>
+        </is>
+      </c>
+      <c r="B234" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C234" s="7" t="inlineStr">
+        <is>
+          <t>Bát tô canh vẽ tay</t>
+        </is>
+      </c>
+      <c r="D234" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E234" s="8" t="inlineStr"/>
+      <c r="F234" s="7" t="inlineStr">
+        <is>
+          <t>Men lam vẽ vàng</t>
+        </is>
+      </c>
+      <c r="G234" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H234" s="9" t="n"/>
+      <c r="I234" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay; PDF ghi giá 0 – để trống, cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="J234" s="8" t="inlineStr">
+        <is>
+          <t>Ngừng dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="7" t="inlineStr">
+        <is>
+          <t>DA08-ML</t>
+        </is>
+      </c>
+      <c r="B235" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C235" s="7" t="inlineStr">
+        <is>
+          <t>Đĩa cánh vẽ tay</t>
+        </is>
+      </c>
+      <c r="D235" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E235" s="8" t="inlineStr"/>
+      <c r="F235" s="7" t="inlineStr">
+        <is>
+          <t>Men lam</t>
+        </is>
+      </c>
+      <c r="G235" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H235" s="9" t="n">
+        <v>132000</v>
+      </c>
+      <c r="I235" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+      <c r="J235" s="8" t="inlineStr">
+        <is>
+          <t>Đang dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="7" t="inlineStr">
+        <is>
+          <t>DA08-VV</t>
+        </is>
+      </c>
+      <c r="B236" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C236" s="7" t="inlineStr">
+        <is>
+          <t>Đĩa cánh vẽ tay</t>
+        </is>
+      </c>
+      <c r="D236" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E236" s="8" t="inlineStr"/>
+      <c r="F236" s="7" t="inlineStr">
+        <is>
+          <t>Men lam vẽ vàng</t>
+        </is>
+      </c>
+      <c r="G236" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H236" s="9" t="n"/>
+      <c r="I236" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay; PDF ghi giá 0 – để trống, cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="J236" s="8" t="inlineStr">
+        <is>
+          <t>Ngừng dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="7" t="inlineStr">
+        <is>
+          <t>DA09-ML</t>
+        </is>
+      </c>
+      <c r="B237" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C237" s="7" t="inlineStr">
+        <is>
+          <t>Bát cơm vẽ tay</t>
+        </is>
+      </c>
+      <c r="D237" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E237" s="8" t="inlineStr"/>
+      <c r="F237" s="7" t="inlineStr">
+        <is>
+          <t>Men lam</t>
+        </is>
+      </c>
+      <c r="G237" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H237" s="9" t="n">
+        <v>66000</v>
+      </c>
+      <c r="I237" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+      <c r="J237" s="8" t="inlineStr">
+        <is>
+          <t>Đang dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="7" t="inlineStr">
+        <is>
+          <t>DA09-VV</t>
+        </is>
+      </c>
+      <c r="B238" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C238" s="7" t="inlineStr">
+        <is>
+          <t>Bát cơm vẽ tay</t>
+        </is>
+      </c>
+      <c r="D238" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E238" s="8" t="inlineStr"/>
+      <c r="F238" s="7" t="inlineStr">
+        <is>
+          <t>Men lam vẽ vàng</t>
+        </is>
+      </c>
+      <c r="G238" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H238" s="9" t="n"/>
+      <c r="I238" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay; PDF ghi giá 0 – để trống, cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="J238" s="8" t="inlineStr">
+        <is>
+          <t>Ngừng dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="7" t="inlineStr">
+        <is>
+          <t>DA10-ML</t>
+        </is>
+      </c>
+      <c r="B239" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t>Bát mắm, muối vẽ tay</t>
+        </is>
+      </c>
+      <c r="D239" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E239" s="8" t="inlineStr"/>
+      <c r="F239" s="7" t="inlineStr">
+        <is>
+          <t>Men lam</t>
+        </is>
+      </c>
+      <c r="G239" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H239" s="9" t="n">
+        <v>52800</v>
+      </c>
+      <c r="I239" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+      <c r="J239" s="8" t="inlineStr">
+        <is>
+          <t>Đang dùng</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="7" t="inlineStr">
+        <is>
+          <t>DA10-VV</t>
+        </is>
+      </c>
+      <c r="B240" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C240" s="7" t="inlineStr">
+        <is>
+          <t>Bát mắm, muối vẽ tay</t>
+        </is>
+      </c>
+      <c r="D240" s="8" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E240" s="8" t="inlineStr"/>
+      <c r="F240" s="7" t="inlineStr">
+        <is>
+          <t>Men lam vẽ vàng</t>
+        </is>
+      </c>
+      <c r="G240" s="8" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="H240" s="9" t="n"/>
+      <c r="I240" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay; PDF ghi giá 0 – để trống, cần kiểm tra</t>
+        </is>
+      </c>
+      <c r="J240" s="8" t="inlineStr">
+        <is>
+          <t>Ngừng dùng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J232"/>
+  <autoFilter ref="A4:J240"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11698,7 +12058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11789,10 +12149,10 @@
         </is>
       </c>
       <c r="G2" s="10" t="n">
-        <v>19000000</v>
+        <v>23000000</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>38800000</v>
+        <v>38600000</v>
       </c>
       <c r="I2" s="7" t="inlineStr"/>
     </row>
@@ -11822,7 +12182,7 @@
         </is>
       </c>
       <c r="G3" s="10" t="n">
-        <v>17500000</v>
+        <v>21500000</v>
       </c>
       <c r="H3" s="10" t="n">
         <v>36500000</v>
@@ -11855,7 +12215,7 @@
         </is>
       </c>
       <c r="G4" s="10" t="n">
-        <v>11000000</v>
+        <v>13500000</v>
       </c>
       <c r="H4" s="10" t="n">
         <v>21000000</v>
@@ -11892,10 +12252,10 @@
         </is>
       </c>
       <c r="G5" s="10" t="n">
-        <v>16500000</v>
+        <v>20500000</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>37500000</v>
+        <v>37600000</v>
       </c>
       <c r="I5" s="7" t="inlineStr"/>
     </row>
@@ -11925,7 +12285,7 @@
         </is>
       </c>
       <c r="G6" s="10" t="n">
-        <v>15500000</v>
+        <v>19000000</v>
       </c>
       <c r="H6" s="10" t="n">
         <v>35500000</v>
@@ -11958,7 +12318,7 @@
         </is>
       </c>
       <c r="G7" s="10" t="n">
-        <v>8800000</v>
+        <v>11000000</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>20000000</v>
@@ -11987,7 +12347,7 @@
         </is>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1100000</v>
+        <v>1500000</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>2100000</v>
@@ -12028,7 +12388,7 @@
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>6600000</v>
+        <v>8000000</v>
       </c>
       <c r="H9" s="10" t="n">
         <v>15500000</v>
@@ -12069,7 +12429,7 @@
         </is>
       </c>
       <c r="G10" s="10" t="n">
-        <v>2640000</v>
+        <v>3000000</v>
       </c>
       <c r="H10" s="10" t="n">
         <v>6600000</v>
@@ -12106,7 +12466,7 @@
         </is>
       </c>
       <c r="G11" s="10" t="n">
-        <v>2200000</v>
+        <v>2650000</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>5300000</v>
@@ -12143,7 +12503,7 @@
         </is>
       </c>
       <c r="G12" s="10" t="n">
-        <v>1200000</v>
+        <v>1450000</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>3700000</v>
@@ -12184,7 +12544,7 @@
         </is>
       </c>
       <c r="G13" s="10" t="n">
-        <v>700000</v>
+        <v>850000</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>2500000</v>
@@ -12225,7 +12585,7 @@
         </is>
       </c>
       <c r="G14" s="10" t="n">
-        <v>550000</v>
+        <v>660000</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>2200000</v>
@@ -12266,7 +12626,7 @@
         </is>
       </c>
       <c r="G15" s="10" t="n">
-        <v>440000</v>
+        <v>530000</v>
       </c>
       <c r="H15" s="10" t="n">
         <v>1900000</v>
@@ -12307,7 +12667,7 @@
         </is>
       </c>
       <c r="G16" s="10" t="n">
-        <v>400000</v>
+        <v>480000</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>1750000</v>
@@ -12348,7 +12708,7 @@
         </is>
       </c>
       <c r="G17" s="10" t="n">
-        <v>265000</v>
+        <v>320000</v>
       </c>
       <c r="H17" s="10" t="n">
         <v>1450000</v>
@@ -12389,7 +12749,7 @@
         </is>
       </c>
       <c r="G18" s="10" t="n">
-        <v>210000</v>
+        <v>250000</v>
       </c>
       <c r="H18" s="10" t="n">
         <v>1200000</v>
@@ -12430,7 +12790,7 @@
         </is>
       </c>
       <c r="G19" s="10" t="n">
-        <v>2200000</v>
+        <v>2650000</v>
       </c>
       <c r="H19" s="10" t="n">
         <v>3800000</v>
@@ -12471,7 +12831,7 @@
         </is>
       </c>
       <c r="G20" s="10" t="n">
-        <v>1000000</v>
+        <v>1200000</v>
       </c>
       <c r="H20" s="10" t="n">
         <v>2500000</v>
@@ -12512,7 +12872,7 @@
         </is>
       </c>
       <c r="G21" s="10" t="n">
-        <v>800000</v>
+        <v>960000</v>
       </c>
       <c r="H21" s="10" t="n">
         <v>2300000</v>
@@ -12553,7 +12913,7 @@
         </is>
       </c>
       <c r="G22" s="10" t="n">
-        <v>550000</v>
+        <v>660000</v>
       </c>
       <c r="H22" s="10" t="n">
         <v>2000000</v>
@@ -12594,7 +12954,7 @@
         </is>
       </c>
       <c r="G23" s="10" t="n">
-        <v>450000</v>
+        <v>550000</v>
       </c>
       <c r="H23" s="10" t="n">
         <v>1850000</v>
@@ -12635,7 +12995,7 @@
         </is>
       </c>
       <c r="G24" s="10" t="n">
-        <v>350000</v>
+        <v>420000</v>
       </c>
       <c r="H24" s="10" t="n">
         <v>1600000</v>
@@ -12676,7 +13036,7 @@
         </is>
       </c>
       <c r="G25" s="10" t="n">
-        <v>1100000</v>
+        <v>1320000</v>
       </c>
       <c r="H25" s="10" t="n">
         <v>3500000</v>
@@ -12717,7 +13077,7 @@
         </is>
       </c>
       <c r="G26" s="10" t="n">
-        <v>650000</v>
+        <v>780000</v>
       </c>
       <c r="H26" s="10" t="n">
         <v>3500000</v>
@@ -12758,7 +13118,7 @@
         </is>
       </c>
       <c r="G27" s="10" t="n">
-        <v>510000</v>
+        <v>620000</v>
       </c>
       <c r="H27" s="10" t="n">
         <v>2100000</v>
@@ -12799,7 +13159,7 @@
         </is>
       </c>
       <c r="G28" s="10" t="n">
-        <v>400000</v>
+        <v>480000</v>
       </c>
       <c r="H28" s="10" t="n">
         <v>1800000</v>
@@ -12840,7 +13200,7 @@
         </is>
       </c>
       <c r="G29" s="10" t="n">
-        <v>310000</v>
+        <v>380000</v>
       </c>
       <c r="H29" s="10" t="n">
         <v>1600000</v>
@@ -12881,7 +13241,7 @@
         </is>
       </c>
       <c r="G30" s="10" t="n">
-        <v>230000</v>
+        <v>280000</v>
       </c>
       <c r="H30" s="10" t="n">
         <v>1400000</v>
@@ -12922,7 +13282,7 @@
         </is>
       </c>
       <c r="G31" s="10" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="H31" s="10" t="n">
         <v>1150000</v>
@@ -12963,7 +13323,7 @@
         </is>
       </c>
       <c r="G32" s="10" t="n">
-        <v>2100000</v>
+        <v>2500000</v>
       </c>
       <c r="H32" s="10" t="n">
         <v>3500000</v>
@@ -13004,7 +13364,7 @@
         </is>
       </c>
       <c r="G33" s="10" t="n">
-        <v>880000</v>
+        <v>1100000</v>
       </c>
       <c r="H33" s="10" t="n">
         <v>2500000</v>
@@ -13045,7 +13405,7 @@
         </is>
       </c>
       <c r="G34" s="10" t="n">
-        <v>770000</v>
+        <v>930000</v>
       </c>
       <c r="H34" s="10" t="n">
         <v>2200000</v>
@@ -13086,7 +13446,7 @@
         </is>
       </c>
       <c r="G35" s="10" t="n">
-        <v>660000</v>
+        <v>800000</v>
       </c>
       <c r="H35" s="10" t="n">
         <v>1900000</v>
@@ -13127,7 +13487,7 @@
         </is>
       </c>
       <c r="G36" s="10" t="n">
-        <v>550000</v>
+        <v>660000</v>
       </c>
       <c r="H36" s="10" t="n">
         <v>1700000</v>
@@ -13168,7 +13528,7 @@
         </is>
       </c>
       <c r="G37" s="10" t="n">
-        <v>270000</v>
+        <v>325000</v>
       </c>
       <c r="H37" s="10" t="n">
         <v>1500000</v>
@@ -13205,7 +13565,7 @@
         </is>
       </c>
       <c r="G38" s="10" t="n">
-        <v>230000</v>
+        <v>280000</v>
       </c>
       <c r="H38" s="10" t="n">
         <v>650000</v>
@@ -13242,7 +13602,7 @@
         </is>
       </c>
       <c r="G39" s="10" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="H39" s="10" t="n">
         <v>750000</v>
@@ -13279,7 +13639,7 @@
         </is>
       </c>
       <c r="G40" s="10" t="n">
-        <v>290000</v>
+        <v>350000</v>
       </c>
       <c r="H40" s="10" t="n">
         <v>850000</v>
@@ -13316,7 +13676,7 @@
         </is>
       </c>
       <c r="G41" s="10" t="n">
-        <v>320000</v>
+        <v>380000</v>
       </c>
       <c r="H41" s="10" t="n">
         <v>950000</v>
@@ -13353,7 +13713,7 @@
         </is>
       </c>
       <c r="G42" s="10" t="n">
-        <v>450000</v>
+        <v>540000</v>
       </c>
       <c r="H42" s="10" t="n">
         <v>1150000</v>
@@ -13390,7 +13750,7 @@
         </is>
       </c>
       <c r="G43" s="10" t="n">
-        <v>480000</v>
+        <v>580000</v>
       </c>
       <c r="H43" s="10" t="n">
         <v>1250000</v>
@@ -13431,7 +13791,7 @@
         </is>
       </c>
       <c r="G44" s="10" t="n">
-        <v>750000</v>
+        <v>900000</v>
       </c>
       <c r="H44" s="10" t="n">
         <v>2750000</v>
@@ -13472,7 +13832,7 @@
         </is>
       </c>
       <c r="G45" s="10" t="n">
-        <v>1050000</v>
+        <v>1250000</v>
       </c>
       <c r="H45" s="10" t="n">
         <v>3200000</v>
@@ -13513,7 +13873,7 @@
         </is>
       </c>
       <c r="G46" s="10" t="n">
-        <v>980000</v>
+        <v>1200000</v>
       </c>
       <c r="H46" s="10" t="n">
         <v>2400000</v>
@@ -13554,7 +13914,7 @@
         </is>
       </c>
       <c r="G47" s="10" t="n">
-        <v>2200000</v>
+        <v>2650000</v>
       </c>
       <c r="H47" s="10" t="n">
         <v>4200000</v>
@@ -13595,7 +13955,7 @@
         </is>
       </c>
       <c r="G48" s="10" t="n">
-        <v>3300000</v>
+        <v>4000000</v>
       </c>
       <c r="H48" s="10" t="n">
         <v>6300000</v>
@@ -13636,7 +13996,7 @@
         </is>
       </c>
       <c r="G49" s="10" t="n">
-        <v>350000</v>
+        <v>420000</v>
       </c>
       <c r="H49" s="10" t="n">
         <v>1400000</v>
@@ -13677,7 +14037,7 @@
         </is>
       </c>
       <c r="G50" s="10" t="n">
-        <v>280000</v>
+        <v>340000</v>
       </c>
       <c r="H50" s="10" t="n">
         <v>1200000</v>
@@ -13718,7 +14078,7 @@
         </is>
       </c>
       <c r="G51" s="10" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="H51" s="10" t="n">
         <v>950000</v>
@@ -13759,7 +14119,7 @@
         </is>
       </c>
       <c r="G52" s="10" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="H52" s="10" t="n">
         <v>750000</v>
@@ -13800,7 +14160,7 @@
         </is>
       </c>
       <c r="G53" s="10" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="H53" s="10" t="n">
         <v>1050000</v>
@@ -13841,7 +14201,7 @@
         </is>
       </c>
       <c r="G54" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H54" s="10" t="n">
         <v>900000</v>
@@ -13882,7 +14242,7 @@
         </is>
       </c>
       <c r="G55" s="10" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="H55" s="10" t="n">
         <v>780000</v>
@@ -13923,7 +14283,7 @@
         </is>
       </c>
       <c r="G56" s="10" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="H56" s="10" t="n">
         <v>680000</v>
@@ -13964,7 +14324,7 @@
         </is>
       </c>
       <c r="G57" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H57" s="10" t="n">
         <v>850000</v>
@@ -14005,7 +14365,7 @@
         </is>
       </c>
       <c r="G58" s="10" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="H58" s="10" t="n">
         <v>750000</v>
@@ -14046,7 +14406,7 @@
         </is>
       </c>
       <c r="G59" s="10" t="n">
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="H59" s="10" t="n">
         <v>650000</v>
@@ -14087,7 +14447,7 @@
         </is>
       </c>
       <c r="G60" s="10" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="H60" s="10" t="n">
         <v>600000</v>
@@ -14128,7 +14488,7 @@
         </is>
       </c>
       <c r="G61" s="10" t="n">
-        <v>910000</v>
+        <v>1100000</v>
       </c>
       <c r="H61" s="10" t="n">
         <v>1800000</v>
@@ -14169,7 +14529,7 @@
         </is>
       </c>
       <c r="G62" s="10" t="n">
-        <v>785000</v>
+        <v>950000</v>
       </c>
       <c r="H62" s="10" t="n">
         <v>1600000</v>
@@ -14210,7 +14570,7 @@
         </is>
       </c>
       <c r="G63" s="10" t="n">
-        <v>660000</v>
+        <v>800000</v>
       </c>
       <c r="H63" s="10" t="n">
         <v>1500000</v>
@@ -14251,7 +14611,7 @@
         </is>
       </c>
       <c r="G64" s="10" t="n">
-        <v>575000</v>
+        <v>700000</v>
       </c>
       <c r="H64" s="10" t="n">
         <v>1350000</v>
@@ -14292,7 +14652,7 @@
         </is>
       </c>
       <c r="G65" s="10" t="n">
-        <v>450000</v>
+        <v>550000</v>
       </c>
       <c r="H65" s="10" t="n">
         <v>1200000</v>
@@ -14333,7 +14693,7 @@
         </is>
       </c>
       <c r="G66" s="10" t="n">
-        <v>330000</v>
+        <v>400000</v>
       </c>
       <c r="H66" s="10" t="n">
         <v>1100000</v>
@@ -14374,7 +14734,7 @@
         </is>
       </c>
       <c r="G67" s="10" t="n">
-        <v>280000</v>
+        <v>350000</v>
       </c>
       <c r="H67" s="10" t="n">
         <v>1000000</v>
@@ -14415,7 +14775,7 @@
         </is>
       </c>
       <c r="G68" s="10" t="n">
-        <v>240000</v>
+        <v>300000</v>
       </c>
       <c r="H68" s="10" t="n">
         <v>750000</v>
@@ -14456,7 +14816,7 @@
         </is>
       </c>
       <c r="G69" s="10" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="H69" s="10" t="n">
         <v>650000</v>
@@ -14497,7 +14857,7 @@
         </is>
       </c>
       <c r="G70" s="10" t="n">
-        <v>1050000</v>
+        <v>1260000</v>
       </c>
       <c r="H70" s="10" t="n">
         <v>2000000</v>
@@ -14538,7 +14898,7 @@
         </is>
       </c>
       <c r="G71" s="10" t="n">
-        <v>890000</v>
+        <v>1100000</v>
       </c>
       <c r="H71" s="10" t="n">
         <v>1700000</v>
@@ -14579,7 +14939,7 @@
         </is>
       </c>
       <c r="G72" s="10" t="n">
-        <v>750000</v>
+        <v>900000</v>
       </c>
       <c r="H72" s="10" t="n">
         <v>1500000</v>
@@ -14620,7 +14980,7 @@
         </is>
       </c>
       <c r="G73" s="10" t="n">
-        <v>620000</v>
+        <v>750000</v>
       </c>
       <c r="H73" s="10" t="n">
         <v>1400000</v>
@@ -14661,7 +15021,7 @@
         </is>
       </c>
       <c r="G74" s="10" t="n">
-        <v>490000</v>
+        <v>600000</v>
       </c>
       <c r="H74" s="10" t="n">
         <v>1300000</v>
@@ -14702,7 +15062,7 @@
         </is>
       </c>
       <c r="G75" s="10" t="n">
-        <v>390000</v>
+        <v>480000</v>
       </c>
       <c r="H75" s="10" t="n">
         <v>1100000</v>
@@ -14743,7 +15103,7 @@
         </is>
       </c>
       <c r="G76" s="10" t="n">
-        <v>330000</v>
+        <v>400000</v>
       </c>
       <c r="H76" s="10" t="n">
         <v>1000000</v>
@@ -14784,7 +15144,7 @@
         </is>
       </c>
       <c r="G77" s="10" t="n">
-        <v>260000</v>
+        <v>320000</v>
       </c>
       <c r="H77" s="10" t="n">
         <v>850000</v>
@@ -14821,7 +15181,7 @@
         </is>
       </c>
       <c r="G78" s="10" t="n">
-        <v>120000</v>
+        <v>150000</v>
       </c>
       <c r="H78" s="10" t="n">
         <v>750000</v>
@@ -14858,7 +15218,7 @@
         </is>
       </c>
       <c r="G79" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H79" s="10" t="n">
         <v>980000</v>
@@ -14895,7 +15255,7 @@
         </is>
       </c>
       <c r="G80" s="10" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="H80" s="10" t="n">
         <v>850000</v>
@@ -14932,7 +15292,7 @@
         </is>
       </c>
       <c r="G81" s="10" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="H81" s="10" t="n">
         <v>1050000</v>
@@ -14969,7 +15329,7 @@
         </is>
       </c>
       <c r="G82" s="10" t="n">
-        <v>20000</v>
+        <v>25000</v>
       </c>
       <c r="H82" s="10" t="n">
         <v>105000</v>
@@ -15010,7 +15370,7 @@
         </is>
       </c>
       <c r="G83" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H83" s="10" t="n">
         <v>680000</v>
@@ -15051,7 +15411,7 @@
         </is>
       </c>
       <c r="G84" s="10" t="n">
-        <v>150000</v>
+        <v>180000</v>
       </c>
       <c r="H84" s="10" t="n">
         <v>600000</v>
@@ -15092,7 +15452,7 @@
         </is>
       </c>
       <c r="G85" s="10" t="n">
-        <v>200000</v>
+        <v>240000</v>
       </c>
       <c r="H85" s="10" t="n">
         <v>1000000</v>
@@ -15133,7 +15493,7 @@
         </is>
       </c>
       <c r="G86" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H86" s="10" t="n">
         <v>900000</v>
@@ -15174,7 +15534,7 @@
         </is>
       </c>
       <c r="G87" s="10" t="n">
-        <v>165000</v>
+        <v>200000</v>
       </c>
       <c r="H87" s="10" t="n">
         <v>735000</v>
@@ -15215,7 +15575,7 @@
         </is>
       </c>
       <c r="G88" s="10" t="n">
-        <v>135000</v>
+        <v>165000</v>
       </c>
       <c r="H88" s="10" t="n">
         <v>680000</v>
@@ -15256,7 +15616,7 @@
         </is>
       </c>
       <c r="G89" s="10" t="n">
-        <v>165000</v>
+        <v>200000</v>
       </c>
       <c r="H89" s="10" t="n">
         <v>735000</v>
@@ -15297,7 +15657,7 @@
         </is>
       </c>
       <c r="G90" s="10" t="n">
-        <v>135000</v>
+        <v>160000</v>
       </c>
       <c r="H90" s="10" t="n">
         <v>680000</v>
@@ -15338,7 +15698,7 @@
         </is>
       </c>
       <c r="G91" s="10" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="H91" s="10" t="n">
         <v>880000</v>
@@ -15379,7 +15739,7 @@
         </is>
       </c>
       <c r="G92" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H92" s="10" t="n">
         <v>800000</v>
@@ -15420,7 +15780,7 @@
         </is>
       </c>
       <c r="G93" s="10" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="H93" s="10" t="n">
         <v>780000</v>
@@ -15461,7 +15821,7 @@
         </is>
       </c>
       <c r="G94" s="10" t="n">
-        <v>180000</v>
+        <v>220000</v>
       </c>
       <c r="H94" s="10" t="n">
         <v>680000</v>
@@ -15498,7 +15858,7 @@
         </is>
       </c>
       <c r="G95" s="10" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
       <c r="H95" s="10" t="n">
         <v>780000</v>
@@ -15531,7 +15891,7 @@
         </is>
       </c>
       <c r="G96" s="10" t="n">
-        <v>22000</v>
+        <v>28000</v>
       </c>
       <c r="H96" s="10" t="n">
         <v>0</v>
@@ -15568,7 +15928,7 @@
         </is>
       </c>
       <c r="G97" s="10" t="n">
-        <v>200000</v>
+        <v>270000</v>
       </c>
       <c r="H97" s="10" t="n">
         <v>1000000</v>
@@ -15601,7 +15961,7 @@
         </is>
       </c>
       <c r="G98" s="10" t="n">
-        <v>165000</v>
+        <v>200000</v>
       </c>
       <c r="H98" s="10" t="n">
         <v>800000</v>
@@ -15630,7 +15990,7 @@
         </is>
       </c>
       <c r="G99" s="10" t="n">
-        <v>22000</v>
+        <v>28000</v>
       </c>
       <c r="H99" s="10" t="n">
         <v>320000</v>
@@ -15667,7 +16027,7 @@
         </is>
       </c>
       <c r="G100" s="10" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="H100" s="10" t="n">
         <v>85000</v>
@@ -15708,7 +16068,7 @@
         </is>
       </c>
       <c r="G101" s="10" t="n">
-        <v>88000</v>
+        <v>110000</v>
       </c>
       <c r="H101" s="10" t="n">
         <v>380000</v>
@@ -15749,7 +16109,7 @@
         </is>
       </c>
       <c r="G102" s="10" t="n">
-        <v>66000</v>
+        <v>80000</v>
       </c>
       <c r="H102" s="10" t="n">
         <v>370000</v>
@@ -15786,7 +16146,7 @@
         </is>
       </c>
       <c r="G103" s="10" t="n">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="H103" s="10" t="n">
         <v>360000</v>
@@ -15823,7 +16183,7 @@
         </is>
       </c>
       <c r="G104" s="10" t="n">
-        <v>265000</v>
+        <v>320000</v>
       </c>
       <c r="H104" s="10" t="n">
         <v>1400000</v>
@@ -15856,7 +16216,7 @@
         </is>
       </c>
       <c r="G105" s="10" t="n">
-        <v>400000</v>
+        <v>480000</v>
       </c>
       <c r="H105" s="10" t="n">
         <v>1700000</v>
@@ -15885,7 +16245,7 @@
         </is>
       </c>
       <c r="G106" s="10" t="n">
-        <v>22000</v>
+        <v>26000</v>
       </c>
       <c r="H106" s="10" t="n">
         <v>320000</v>
@@ -15926,7 +16286,7 @@
         </is>
       </c>
       <c r="G107" s="10" t="n">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="H107" s="10" t="n">
         <v>440000</v>
@@ -15967,7 +16327,7 @@
         </is>
       </c>
       <c r="G108" s="10" t="n">
-        <v>88000</v>
+        <v>105000</v>
       </c>
       <c r="H108" s="10" t="n">
         <v>380000</v>
@@ -16008,7 +16368,7 @@
         </is>
       </c>
       <c r="G109" s="10" t="n">
-        <v>66000</v>
+        <v>80000</v>
       </c>
       <c r="H109" s="10" t="n">
         <v>320000</v>
@@ -16045,7 +16405,7 @@
         </is>
       </c>
       <c r="G110" s="10" t="n">
-        <v>45000</v>
+        <v>55000</v>
       </c>
       <c r="H110" s="10" t="n">
         <v>295000</v>
@@ -16086,7 +16446,7 @@
         </is>
       </c>
       <c r="G111" s="10" t="n">
-        <v>1650000</v>
+        <v>2000000</v>
       </c>
       <c r="H111" s="10" t="n">
         <v>6300000</v>
@@ -16127,7 +16487,7 @@
         </is>
       </c>
       <c r="G112" s="10" t="n">
-        <v>1320000</v>
+        <v>1600000</v>
       </c>
       <c r="H112" s="10" t="n">
         <v>4300000</v>
@@ -16164,7 +16524,7 @@
         </is>
       </c>
       <c r="G113" s="10" t="n">
-        <v>660000</v>
+        <v>800000</v>
       </c>
       <c r="H113" s="10" t="n">
         <v>1350000</v>
@@ -16197,7 +16557,7 @@
         </is>
       </c>
       <c r="G114" s="10" t="n">
-        <v>220000</v>
+        <v>265000</v>
       </c>
       <c r="H114" s="10" t="n">
         <v>1050000</v>
@@ -16226,12 +16586,160 @@
         </is>
       </c>
       <c r="G115" s="10" t="n">
-        <v>135000</v>
+        <v>160000</v>
       </c>
       <c r="H115" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I115" s="7" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>Bát tô canh vẽ tay</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr"/>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="G116" s="10" t="n">
+        <v>686400</v>
+      </c>
+      <c r="H116" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>Đĩa cánh vẽ tay</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr"/>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="G117" s="10" t="n">
+        <v>132000</v>
+      </c>
+      <c r="H117" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I117" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>Bát cơm vẽ tay</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr"/>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="G118" s="10" t="n">
+        <v>66000</v>
+      </c>
+      <c r="H118" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I118" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>Bộ đồ ăn cúng</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>Bát mắm, muối vẽ tay</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>Sen</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr"/>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>chiếc</t>
+        </is>
+      </c>
+      <c r="G119" s="10" t="n">
+        <v>52800</v>
+      </c>
+      <c r="H119" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I119" s="7" t="inlineStr">
+        <is>
+          <t>Lẻ từ bộ HMT sen vẽ tay</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>